<commit_message>
chore: update weekly grant snapshot
</commit_message>
<xml_diff>
--- a/state/daysee_grants_delta_latest.xlsx
+++ b/state/daysee_grants_delta_latest.xlsx
@@ -61,10 +61,10 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -434,11 +434,11 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>metric</t>
@@ -450,66 +450,66 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>run_type</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>delta_run</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
+          <t>current_count</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>current_count</t>
+          <t>previous_count</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
         <v>8</v>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1">
+    <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>previous_count</t>
+          <t>new_count</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" ht="18" customHeight="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>new_count</t>
+          <t>updated_count</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>removed_count</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>updated_count</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" ht="18" customHeight="1">
+    <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>removed_count</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>0</v>
+          <t>generated_at</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-25 20:19:17</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -526,29 +526,29 @@
   <dimension ref="A1:T1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="34" customWidth="1" min="13" max="13"/>
-    <col width="28" customWidth="1" min="14" max="14"/>
-    <col width="34" customWidth="1" min="15" max="15"/>
-    <col width="22" customWidth="1" min="16" max="16"/>
-    <col width="34" customWidth="1" min="17" max="17"/>
-    <col width="22" customWidth="1" min="18" max="18"/>
-    <col width="24" customWidth="1" min="19" max="19"/>
-    <col width="34" customWidth="1" min="20" max="20"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="23" customWidth="1" min="16" max="16"/>
+    <col width="29" customWidth="1" min="17" max="17"/>
+    <col width="27" customWidth="1" min="18" max="18"/>
+    <col width="21" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>title</t>
@@ -661,33 +661,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U9"/>
+  <dimension ref="A1:T8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="34" customWidth="1" min="13" max="13"/>
-    <col width="28" customWidth="1" min="14" max="14"/>
-    <col width="34" customWidth="1" min="15" max="15"/>
-    <col width="22" customWidth="1" min="16" max="16"/>
-    <col width="34" customWidth="1" min="17" max="17"/>
-    <col width="22" customWidth="1" min="18" max="18"/>
-    <col width="24" customWidth="1" min="19" max="19"/>
-    <col width="34" customWidth="1" min="20" max="20"/>
-    <col width="24" customWidth="1" min="21" max="21"/>
+    <col width="45" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="45" customWidth="1" min="15" max="15"/>
+    <col width="23" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="17" max="17"/>
+    <col width="27" customWidth="1" min="18" max="18"/>
+    <col width="26" customWidth="1" min="19" max="19"/>
+    <col width="43" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>title</t>
@@ -788,26 +787,21 @@
           <t>detail_url</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>changed_fields</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="42" customHeight="1">
+    </row>
+    <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>115年度推動工作與生活平衡補助計畫</t>
+          <t>115年度原住民族促進就業獎勵計畫</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>勞動部</t>
+          <t>原住民族委員會</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>企業</t>
+          <t>企業｜個人</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -822,17 +816,17 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>婦女｜產業發展｜青年</t>
+          <t>原住民｜產業發展</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>婦女</t>
+          <t>原住民</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -840,41 +834,37 @@
           <t>產業發展</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>青年</t>
-        </is>
-      </c>
+      <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=115年度推動工作與生活平衡補助計畫</t>
+          <t>https://www.google.com/search?q=115年度原住民族促進就業獎勵計畫</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>115年度推動工作與生活平衡補助計畫</t>
+          <t>115年度原住民族促進就業獎勵計畫</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>https://www.mol.gov.tw/</t>
+          <t>https://www.cip.gov.tw/</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>www.mol.gov.tw</t>
+          <t>www.cip.gov.tw</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>https://www.mol.gov.tw/</t>
+          <t>https://www.cip.gov.tw/</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>www.mol.gov.tw</t>
+          <t>www.cip.gov.tw</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr">
@@ -884,29 +874,24 @@
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t>https://dayseechat.com/subsidy/grant-446/</t>
-        </is>
-      </c>
-      <c r="U2" s="2" t="inlineStr">
-        <is>
-          <t>plan_source | eligible_targets | applicable_region | grant_amount | organizer_site_url | official_organizer_site_url | official_url_status</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="42" customHeight="1">
+          <t>https://dayseechat.com/subsidy/grant-439/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="36" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>115年度數位服務創新補助計畫</t>
+          <t>115年度推展海內外客家事務交流合作活動補助</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>數位發展部</t>
+          <t>客家委員會</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>企業</t>
+          <t>學校｜民間團體</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -916,27 +901,27 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>100萬以上</t>
+          <t>11萬-50萬</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>產業發展｜創新創業</t>
+          <t>客家｜文化藝文</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>產業發展</t>
+          <t>客家</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>創新創業</t>
+          <t>文化藝文</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
@@ -944,32 +929,32 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=115年度數位服務創新補助計畫</t>
+          <t>https://www.google.com/search?q=115年度推展海內外客家事務交流合作活動補助</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>115年度數位服務創新補助計畫</t>
+          <t>115年度推展海內外客家事務交流合作活動補助</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>https://moda.gov.tw/</t>
+          <t>https://www.hakka.gov.tw/</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>moda.gov.tw</t>
+          <t>www.hakka.gov.tw</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>https://moda.gov.tw/</t>
+          <t>https://www.hakka.gov.tw/</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>moda.gov.tw</t>
+          <t>www.hakka.gov.tw</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
@@ -979,16 +964,11 @@
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>https://dayseechat.com/subsidy/grant-448/</t>
-        </is>
-      </c>
-      <c r="U3" s="2" t="inlineStr">
-        <is>
-          <t>plan_source | eligible_targets | applicable_region | grant_amount | deadline_date | organizer_site_url | official_organizer_site_url | official_url_status</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="42" customHeight="1">
+          <t>https://dayseechat.com/subsidy/grant-437/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>115年臺中市農業作物類生產設備設施改善補助計畫</t>
@@ -1001,7 +981,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>企業 個人 民間團體</t>
+          <t>企業｜個人｜民間團體</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1077,26 +1057,21 @@
           <t>https://dayseechat.com/subsidy/grant-447/</t>
         </is>
       </c>
-      <c r="U4" s="2" t="inlineStr">
-        <is>
-          <t>plan_source | eligible_targets | applicable_region | grant_amount | deadline_date | deadline_text</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="42" customHeight="1">
+    </row>
+    <row r="5" ht="36" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>115年度推動工作與生活平衡補助計畫</t>
+          <t>115年度數位服務創新補助計畫</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>勞動部</t>
+          <t>數位發展部</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>企業 民間團體</t>
+          <t>企業</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1106,22 +1081,22 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>不分金額</t>
+          <t>100萬以上</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>婦女｜產業發展</t>
+          <t>創新創業｜產業發展</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>婦女</t>
+          <t>創新創業</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -1134,64 +1109,59 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=115年度推動工作與生活平衡補助計畫</t>
+          <t>https://www.google.com/search?q=115年度數位服務創新補助計畫</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
+          <t>115年度數位服務創新補助計畫</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>https://moda.gov.tw/</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>moda.gov.tw</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>https://moda.gov.tw/</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>moda.gov.tw</t>
+        </is>
+      </c>
+      <c r="S5" s="2" t="inlineStr">
+        <is>
+          <t>verified_portal_homepage</t>
+        </is>
+      </c>
+      <c r="T5" s="2" t="inlineStr">
+        <is>
+          <t>https://dayseechat.com/subsidy/grant-448/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
           <t>115年度推動工作與生活平衡補助計畫</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mol.gov.tw/</t>
-        </is>
-      </c>
-      <c r="P5" s="2" t="inlineStr">
-        <is>
-          <t>www.mol.gov.tw</t>
-        </is>
-      </c>
-      <c r="Q5" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mol.gov.tw/</t>
-        </is>
-      </c>
-      <c r="R5" s="2" t="inlineStr">
-        <is>
-          <t>www.mol.gov.tw</t>
-        </is>
-      </c>
-      <c r="S5" s="2" t="inlineStr">
-        <is>
-          <t>verified_portal_homepage</t>
-        </is>
-      </c>
-      <c r="T5" s="2" t="inlineStr">
-        <is>
-          <t>https://dayseechat.com/subsidy/grant-438/</t>
-        </is>
-      </c>
-      <c r="U5" s="2" t="inlineStr">
-        <is>
-          <t>plan_source | eligible_targets | applicable_region | grant_amount | deadline_text | organizer_site_url | official_organizer_site_url | official_url_status</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>115年度推展海內外客家事務交流合作活動補助</t>
-        </is>
-      </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>客家委員會</t>
+          <t>勞動部</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>學校 民間團體</t>
+          <t>企業｜民間團體</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -1201,27 +1171,27 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>11萬-50萬</t>
+          <t>不分金額</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>客家｜文化藝文</t>
+          <t>婦女｜產業發展</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>客家</t>
+          <t>婦女</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>文化藝文</t>
+          <t>產業發展</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
@@ -1229,32 +1199,32 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=115年度推展海內外客家事務交流合作活動補助</t>
+          <t>https://www.google.com/search?q=115年度推動工作與生活平衡補助計畫</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>115年度推展海內外客家事務交流合作活動補助</t>
+          <t>115年度推動工作與生活平衡補助計畫</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>https://www.hakka.gov.tw/chhakka/index</t>
+          <t>https://www.mol.gov.tw/</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>www.hakka.gov.tw</t>
+          <t>www.mol.gov.tw</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>https://www.hakka.gov.tw/chhakka/index</t>
+          <t>https://www.mol.gov.tw/</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>www.hakka.gov.tw</t>
+          <t>www.mol.gov.tw</t>
         </is>
       </c>
       <c r="S6" s="2" t="inlineStr">
@@ -1264,59 +1234,54 @@
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>https://dayseechat.com/subsidy/grant-437/</t>
-        </is>
-      </c>
-      <c r="U6" s="2" t="inlineStr">
-        <is>
-          <t>plan_source | eligible_targets | applicable_region | grant_amount | deadline_text | organizer_site_url | official_organizer_site_url | official_url_status</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="42" customHeight="1">
+          <t>https://dayseechat.com/subsidy/grant-438/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>115年度原住民族促進就業獎勵計畫</t>
+          <t>115年臺北市住宅社區創能儲能及節能補助計畫</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>原住民族委員會</t>
+          <t>縣市政府</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>企業 個人</t>
+          <t>個人｜其他對象｜民間團體</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>不分縣市</t>
+          <t>台北</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>不分金額</t>
+          <t>51萬-100萬</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>產業發展｜原住民</t>
+          <t>生態環境｜社區議題</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>產業發展</t>
+          <t>生態環境</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>原住民</t>
+          <t>社區議題</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr"/>
@@ -1324,32 +1289,32 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=115年度原住民族促進就業獎勵計畫</t>
+          <t>https://www.google.com/search?q=115年臺北市住宅社區創能儲能及節能補助計畫</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>115年度原住民族促進就業獎勵計畫</t>
+          <t>115年臺北市住宅社區創能儲能及節能補助計畫</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>https://www.cip.gov.tw/zh-tw/index.html</t>
+          <t>https://www.gov.taipei/</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>www.cip.gov.tw</t>
+          <t>www.gov.taipei</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>https://www.cip.gov.tw/zh-tw/index.html</t>
+          <t>https://www.gov.taipei/</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>www.cip.gov.tw</t>
+          <t>www.gov.taipei</t>
         </is>
       </c>
       <c r="S7" s="2" t="inlineStr">
@@ -1359,19 +1324,14 @@
       </c>
       <c r="T7" s="2" t="inlineStr">
         <is>
-          <t>https://dayseechat.com/subsidy/grant-439/</t>
-        </is>
-      </c>
-      <c r="U7" s="2" t="inlineStr">
-        <is>
-          <t>plan_source | eligible_targets | applicable_region | grant_amount | deadline_date | deadline_text | organizer_site_url | official_organizer_site_url | official_url_status</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="42" customHeight="1">
+          <t>https://dayseechat.com/subsidy/grant-440/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>115年臺北市住宅社區創能儲能及節能補助計畫</t>
+          <t>115年度補助原住民參加國家考試實施計畫</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1381,176 +1341,68 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>個人 其他對象 民間團體</t>
+          <t>個人</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>台北</t>
+          <t>台中</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>51萬-100萬</t>
+          <t>10萬以下</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>生態環境｜社區議題</t>
+          <t>原住民</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>生態環境</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>社區議題</t>
-        </is>
-      </c>
+          <t>原住民</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=115年臺北市住宅社區創能儲能及節能補助計畫</t>
+          <t>https://www.google.com/search?q=115年度補助原住民參加國家考試實施計畫</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>115年臺北市住宅社區創能儲能及節能補助計畫</t>
+          <t>115年度補助原住民參加國家考試實施計畫</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>https://www.gov.taipei/</t>
+          <t>https://www.google.com/search?q=115年度補助原住民參加國家考試實施計畫</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>www.gov.taipei</t>
-        </is>
-      </c>
-      <c r="Q8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.gov.taipei/</t>
-        </is>
-      </c>
-      <c r="R8" s="2" t="inlineStr">
-        <is>
-          <t>www.gov.taipei</t>
-        </is>
-      </c>
+          <t>www.google.com</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr"/>
+      <c r="R8" s="2" t="inlineStr"/>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>verified_portal_homepage</t>
+          <t>bing_title_no_match</t>
         </is>
       </c>
       <c r="T8" s="2" t="inlineStr">
         <is>
-          <t>https://dayseechat.com/subsidy/grant-440/</t>
-        </is>
-      </c>
-      <c r="U8" s="2" t="inlineStr">
-        <is>
-          <t>plan_source | eligible_targets | applicable_region | grant_amount | deadline_date | deadline_text</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>115年度補助原住民參加國家考試實施計畫</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>縣市政府</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>個人</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>台中</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>10萬以下</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-30</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>原住民</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>原住民</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.google.com/search?q=115年度補助原住民參加國家考試實施計畫</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>115年度補助原住民參加國家考試實施計畫</t>
-        </is>
-      </c>
-      <c r="O9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.taichung.gov.tw/</t>
-        </is>
-      </c>
-      <c r="P9" s="2" t="inlineStr">
-        <is>
-          <t>www.taichung.gov.tw</t>
-        </is>
-      </c>
-      <c r="Q9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.taichung.gov.tw/</t>
-        </is>
-      </c>
-      <c r="R9" s="2" t="inlineStr">
-        <is>
-          <t>www.taichung.gov.tw</t>
-        </is>
-      </c>
-      <c r="S9" s="2" t="inlineStr">
-        <is>
-          <t>verified_portal_homepage</t>
-        </is>
-      </c>
-      <c r="T9" s="2" t="inlineStr">
-        <is>
           <t>https://dayseechat.com/subsidy/grant-441/</t>
-        </is>
-      </c>
-      <c r="U9" s="2" t="inlineStr">
-        <is>
-          <t>plan_source | eligible_targets | applicable_region | grant_amount | deadline_date | deadline_text | organizer_site_url | official_organizer_site_url | official_url_status</t>
         </is>
       </c>
     </row>
@@ -1568,29 +1420,29 @@
   <dimension ref="A1:T1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="34" customWidth="1" min="13" max="13"/>
-    <col width="28" customWidth="1" min="14" max="14"/>
-    <col width="34" customWidth="1" min="15" max="15"/>
-    <col width="22" customWidth="1" min="16" max="16"/>
-    <col width="34" customWidth="1" min="17" max="17"/>
-    <col width="22" customWidth="1" min="18" max="18"/>
-    <col width="24" customWidth="1" min="19" max="19"/>
-    <col width="34" customWidth="1" min="20" max="20"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="23" customWidth="1" min="16" max="16"/>
+    <col width="29" customWidth="1" min="17" max="17"/>
+    <col width="27" customWidth="1" min="18" max="18"/>
+    <col width="21" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>title</t>

</xml_diff>

<commit_message>
chore: update weekly grant state
</commit_message>
<xml_diff>
--- a/state/daysee_grants_delta_latest.xlsx
+++ b/state/daysee_grants_delta_latest.xlsx
@@ -473,7 +473,7 @@
         <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0</v>
@@ -622,11 +622,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:S2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="43" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
@@ -638,7 +638,7 @@
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="43" customWidth="1" min="14" max="14"/>
     <col width="23" customWidth="1" min="15" max="15"/>
     <col width="29" customWidth="1" min="16" max="16"/>
     <col width="27" customWidth="1" min="17" max="17"/>
@@ -740,6 +740,71 @@
       <c r="S1" s="1" t="inlineStr">
         <is>
           <t>official_url_confidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>115年度高雄市觀光行銷推廣補助計畫</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>https://dayseechat.com/subsidy/grant-327/</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>縣市政府</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>民間團體</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>10萬以下</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>產業發展</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>https://dayseechat.com/subsidy/grant-327/</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>dayseechat.com</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr"/>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>search_no_match</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
         </is>
       </c>
     </row>

</xml_diff>